<commit_message>
Added project filter + download Excel module with backend routes and frontend integration
</commit_message>
<xml_diff>
--- a/backend/projects.xlsx
+++ b/backend/projects.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -499,9 +499,259 @@
         <v>2025-04-14T07:41:02.444Z</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Starwire Industries</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Certification of Nickel Alloys</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2023-2024</v>
+      </c>
+      <c r="E3">
+        <v>800000</v>
+      </c>
+      <c r="F3">
+        <v>500000</v>
+      </c>
+      <c r="G3" t="str">
+        <v>jay shree ram</v>
+      </c>
+      <c r="H3" t="str">
+        <v xml:space="preserve">om mani padme hum </v>
+      </c>
+      <c r="I3" t="str">
+        <v>Dr John Doe</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Dr Jane Doe</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Dr Rajesh Ganesh</v>
+      </c>
+      <c r="L3" t="str">
+        <v>rajganesh@gmail.com</v>
+      </c>
+      <c r="M3" t="str">
+        <v>1744624304766-bill.pdf</v>
+      </c>
+      <c r="N3" t="str">
+        <v>1744624304767-bill.pdf</v>
+      </c>
+      <c r="O3" t="str">
+        <v>bhuvana@ssn.edu.in</v>
+      </c>
+      <c r="P3" t="str">
+        <v>2025-04-14T09:51:44.774Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ABC Solutions</v>
+      </c>
+      <c r="C4" t="str">
+        <v>AI model solution</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2023-2024</v>
+      </c>
+      <c r="E4">
+        <v>80000</v>
+      </c>
+      <c r="F4">
+        <v>70000</v>
+      </c>
+      <c r="G4" t="str">
+        <v>jay shree ram</v>
+      </c>
+      <c r="H4" t="str">
+        <v>hare ram</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Dr John Doe</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Dr Jane Doe</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Dr Raj</v>
+      </c>
+      <c r="L4" t="str">
+        <v>raj@gmail.com</v>
+      </c>
+      <c r="M4" t="str">
+        <v>1744624399077-bill.pdf</v>
+      </c>
+      <c r="N4" t="str">
+        <v>1744624399077-bill.pdf</v>
+      </c>
+      <c r="O4" t="str">
+        <v>bhuvana@ssn.edu.in</v>
+      </c>
+      <c r="P4" t="str">
+        <v>2025-04-14T09:53:19.081Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v xml:space="preserve">XYZ </v>
+      </c>
+      <c r="C5" t="str">
+        <v>Oil Refinery</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2024-2025</v>
+      </c>
+      <c r="E5">
+        <v>40000</v>
+      </c>
+      <c r="F5">
+        <v>30000</v>
+      </c>
+      <c r="G5" t="str">
+        <v>jay shree ram</v>
+      </c>
+      <c r="H5" t="str">
+        <v>om mani pay mey hun</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Dr John Doe</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Dr Jane Doe</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Dr Murugan</v>
+      </c>
+      <c r="L5" t="str">
+        <v>murugan@gmail.com</v>
+      </c>
+      <c r="M5" t="str">
+        <v>1744624662609-bill.pdf</v>
+      </c>
+      <c r="N5" t="str">
+        <v>1744624662609-bill.pdf</v>
+      </c>
+      <c r="O5" t="str">
+        <v>someone@ssn.edu.in</v>
+      </c>
+      <c r="P5" t="str">
+        <v>2025-04-14T09:57:42.612Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v xml:space="preserve">XYZ </v>
+      </c>
+      <c r="C6" t="str">
+        <v>Oil Refinery</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2024-2025</v>
+      </c>
+      <c r="E6">
+        <v>80000</v>
+      </c>
+      <c r="F6">
+        <v>75000</v>
+      </c>
+      <c r="G6" t="str">
+        <v>jay ram</v>
+      </c>
+      <c r="H6" t="str">
+        <v>om sai ram</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Dr Krishnan</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Dr Radha</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Dr Murugan</v>
+      </c>
+      <c r="L6" t="str">
+        <v>murugan@gmail.com</v>
+      </c>
+      <c r="M6" t="str">
+        <v>1744624709394-bill.pdf</v>
+      </c>
+      <c r="N6" t="str">
+        <v>1744624709394-bill.pdf</v>
+      </c>
+      <c r="O6" t="str">
+        <v>someone@ssn.edu.in</v>
+      </c>
+      <c r="P6" t="str">
+        <v>2025-04-14T09:58:29.398Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v xml:space="preserve">ABC Solutions </v>
+      </c>
+      <c r="C7" t="str">
+        <v>AI model solution</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2024-2025</v>
+      </c>
+      <c r="E7">
+        <v>80000</v>
+      </c>
+      <c r="F7">
+        <v>75000</v>
+      </c>
+      <c r="G7" t="str">
+        <v>om sri</v>
+      </c>
+      <c r="H7" t="str">
+        <v>ram</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Dr Krishnan</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Dr Radha</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Dr Murugan</v>
+      </c>
+      <c r="L7" t="str">
+        <v>murugan@gmail.com</v>
+      </c>
+      <c r="M7" t="str">
+        <v>1744624743610-bill.pdf</v>
+      </c>
+      <c r="N7" t="str">
+        <v>1744624743611-bill.pdf</v>
+      </c>
+      <c r="O7" t="str">
+        <v>someone@ssn.edu.in</v>
+      </c>
+      <c r="P7" t="str">
+        <v>2025-04-14T09:59:03.614Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Final module added: Notifications feature complete
</commit_message>
<xml_diff>
--- a/backend/projects.xlsx
+++ b/backend/projects.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -749,9 +749,59 @@
         <v>2025-04-14T09:59:03.614Z</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v xml:space="preserve">Ganesha industries </v>
+      </c>
+      <c r="C8" t="str">
+        <v>Oil Refinery</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2024-2025</v>
+      </c>
+      <c r="E8">
+        <v>80000</v>
+      </c>
+      <c r="F8">
+        <v>75000</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Ram Sham Sita</v>
+      </c>
+      <c r="H8" t="str">
+        <v>this is project based on certification of oil refinery</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Dr Krishnan</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Dr Radha</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Dr Murugan</v>
+      </c>
+      <c r="L8" t="str">
+        <v>murugan@gmail.com</v>
+      </c>
+      <c r="M8" t="str">
+        <v>1744629327054-bill.pdf</v>
+      </c>
+      <c r="N8" t="str">
+        <v>1744629327054-bill.pdf</v>
+      </c>
+      <c r="O8" t="str">
+        <v>bhuvana@ssn.edu.in</v>
+      </c>
+      <c r="P8" t="str">
+        <v>2025-04-14T11:15:27.061Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>